<commit_message>
Credit limit says what 0 really means; categories show "Parent"; tutorial PDF
- Customer credit limit: the hint said "0 = cash only", but a 0 limit means
  the credit check is skipped (sales/orders.py credit_check). It now says
  "0 = no credit check (a customer who pays cash)" on the form, the API docs
  and the customers Excel template. sales.0005 changes only the help text:
  no SQL.
- Item categories list: the column "Inside" is now "Parent", like the form.
- docs/inventory/INVENTORY-PART1-TUTORIAL.pdf: a 19-page tutorial for the 10
  Inventory pages shown today - every field with what to write, an example
  and what it does in the software (checked against the code), a worked
  example and the messages people may see. Rebuilt with
  docs/scripts/build_inventory_tutorial.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inventory/templates/04-customers.xlsx
+++ b/docs/inventory/templates/04-customers.xlsx
@@ -711,7 +711,7 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>0 = cash only</t>
+          <t>0 = no credit check</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -13073,7 +13073,7 @@
     <dataValidation sqref="C2:C2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Customer type" error="Pick one of: Distributor, Dealer, Retailer, Corporate" prompt="" type="list">
       <formula1>"Distributor,Dealer,Retailer,Corporate"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J2001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Credit limit (BDT)" error="A number, 0 or more." prompt="0 = cash only" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J2:J2001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Credit limit (BDT)" error="A number, 0 or more." prompt="0 = no credit check" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Payment terms (days)" error="A whole number, 0 or more." prompt="" type="whole" operator="greaterThanOrEqual">

</xml_diff>